<commit_message>
Add 集客経路 tally formulas to 設定 tab (per day 8/28-30)
- 設定タブ E/F/G列に日別（28/29/30）の集客経路件数を集計
- 各ルームの集客経路列(E,J,O,T)をCOUNTIFで合算、合計行も追加

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Adod21a7rESEkB4fCREdiE
</commit_message>
<xml_diff>
--- a/ONE'S BODY静岡安倍川店_体験会予約表.xlsx
+++ b/ONE'S BODY静岡安倍川店_体験会予約表.xlsx
@@ -165,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -221,6 +221,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2958,12 +2967,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2977,9 +2988,24 @@
           <t>集客経路リスト</t>
         </is>
       </c>
-      <c r="E1" s="22" t="inlineStr">
-        <is>
-          <t>チェック</t>
+      <c r="D1" s="22" t="inlineStr">
+        <is>
+          <t>集計</t>
+        </is>
+      </c>
+      <c r="E1" s="23" t="inlineStr">
+        <is>
+          <t>8/28</t>
+        </is>
+      </c>
+      <c r="F1" s="23" t="inlineStr">
+        <is>
+          <t>8/29</t>
+        </is>
+      </c>
+      <c r="G1" s="23" t="inlineStr">
+        <is>
+          <t>8/30</t>
         </is>
       </c>
     </row>
@@ -2990,10 +3016,17 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>✅</t>
-        </is>
+      <c r="E2" s="24">
+        <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C2)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C2)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C2)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C2)</f>
+        <v/>
+      </c>
+      <c r="F2" s="24">
+        <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C2)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C2)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C2)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C2)</f>
+        <v/>
+      </c>
+      <c r="G2" s="24">
+        <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C2)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C2)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C2)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C2)</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -3007,6 +3040,18 @@
           <t>Googleマップ</t>
         </is>
       </c>
+      <c r="E3" s="24">
+        <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C3)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C3)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C3)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C3)</f>
+        <v/>
+      </c>
+      <c r="F3" s="24">
+        <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C3)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C3)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C3)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C3)</f>
+        <v/>
+      </c>
+      <c r="G3" s="24">
+        <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C3)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C3)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C3)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C3)</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3019,6 +3064,18 @@
           <t>チラシ</t>
         </is>
       </c>
+      <c r="E4" s="24">
+        <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C4)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C4)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C4)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="24">
+        <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C4)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C4)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C4)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="24">
+        <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C4)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C4)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C4)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C4)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3031,6 +3088,18 @@
           <t>紹介</t>
         </is>
       </c>
+      <c r="E5" s="24">
+        <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C5)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C5)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C5)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="24">
+        <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C5)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C5)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C5)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="24">
+        <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C5)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C5)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C5)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3043,6 +3112,18 @@
           <t>HP</t>
         </is>
       </c>
+      <c r="E6" s="24">
+        <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C6)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C6)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C6)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="24">
+        <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C6)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C6)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C6)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="24">
+        <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C6)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C6)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C6)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C6)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3055,12 +3136,55 @@
           <t>既存会員</t>
         </is>
       </c>
+      <c r="E7" s="24">
+        <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C7)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C7)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C7)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="24">
+        <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C7)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C7)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C7)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="24">
+        <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C7)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C7)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C7)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C7)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="C8" t="inlineStr">
         <is>
           <t>その他</t>
         </is>
+      </c>
+      <c r="E8" s="24">
+        <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C8)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C8)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C8)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="24">
+        <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C8)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C8)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C8)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="24">
+        <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C8)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C8)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C8)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="E9" s="25">
+        <f>SUM(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="25">
+        <f>SUM(F2:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="25">
+        <f>SUM(G2:G8)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 体験者一覧 tab that auto-aggregates trial participants
- 3日分の予約表から氏名の入った枠を縦に自動集約（体験日/氏名/担当者/集客きっかけ）
- E・F列は次回予約有無(〇×)・次回来店日を書式なしで手入力
- Googleスプレッドシート用の集約数式を生成

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Adod21a7rESEkB4fCREdiE
</commit_message>
<xml_diff>
--- a/ONE'S BODY静岡安倍川店_体験会予約表.xlsx
+++ b/ONE'S BODY静岡安倍川店_体験会予約表.xlsx
@@ -10,7 +10,8 @@
     <sheet name="8月28日（金）" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="8月29日（土）" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="8月30日（日）" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="設定" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="体験者一覧" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="設定" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -165,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -219,6 +220,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2963,6 +2967,67 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>体験日</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="inlineStr">
+        <is>
+          <t>氏名</t>
+        </is>
+      </c>
+      <c r="C1" s="22" t="inlineStr">
+        <is>
+          <t>担当者</t>
+        </is>
+      </c>
+      <c r="D1" s="22" t="inlineStr">
+        <is>
+          <t>集客きっかけ</t>
+        </is>
+      </c>
+      <c r="E1" s="22" t="inlineStr">
+        <is>
+          <t>次回予約（〇・×）</t>
+        </is>
+      </c>
+      <c r="F1" s="22" t="inlineStr">
+        <is>
+          <t>次回来店日</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>IFERROR(LET(data,VSTACK(HSTACK(IF('8月28日（金）'!$C$5:$C$22&lt;&gt;"","8/28",""),'8月28日（金）'!$C$5:$C$22,'8月28日（金）'!$B$5:$B$22,'8月28日（金）'!$E$5:$E$22),HSTACK(IF('8月28日（金）'!$H$5:$H$22&lt;&gt;"","8/28",""),'8月28日（金）'!$H$5:$H$22,'8月28日（金）'!$G$5:$G$22,'8月28日（金）'!$J$5:$J$22),HSTACK(IF('8月28日（金）'!$M$5:$M$22&lt;&gt;"","8/28",""),'8月28日（金）'!$M$5:$M$22,'8月28日（金）'!$L$5:$L$22,'8月28日（金）'!$O$5:$O$22),HSTACK(IF('8月28日（金）'!$R$5:$R$22&lt;&gt;"","8/28",""),'8月28日（金）'!$R$5:$R$22,'8月28日（金）'!$Q$5:$Q$22,'8月28日（金）'!$T$5:$T$22),HSTACK(IF('8月29日（土）'!$C$5:$C$22&lt;&gt;"","8/29",""),'8月29日（土）'!$C$5:$C$22,'8月29日（土）'!$B$5:$B$22,'8月29日（土）'!$E$5:$E$22),HSTACK(IF('8月29日（土）'!$H$5:$H$22&lt;&gt;"","8/29",""),'8月29日（土）'!$H$5:$H$22,'8月29日（土）'!$G$5:$G$22,'8月29日（土）'!$J$5:$J$22),HSTACK(IF('8月29日（土）'!$M$5:$M$22&lt;&gt;"","8/29",""),'8月29日（土）'!$M$5:$M$22,'8月29日（土）'!$L$5:$L$22,'8月29日（土）'!$O$5:$O$22),HSTACK(IF('8月29日（土）'!$R$5:$R$22&lt;&gt;"","8/29",""),'8月29日（土）'!$R$5:$R$22,'8月29日（土）'!$Q$5:$Q$22,'8月29日（土）'!$T$5:$T$22),HSTACK(IF('8月30日（日）'!$C$5:$C$22&lt;&gt;"","8/30",""),'8月30日（日）'!$C$5:$C$22,'8月30日（日）'!$B$5:$B$22,'8月30日（日）'!$E$5:$E$22),HSTACK(IF('8月30日（日）'!$H$5:$H$22&lt;&gt;"","8/30",""),'8月30日（日）'!$H$5:$H$22,'8月30日（日）'!$G$5:$G$22,'8月30日（日）'!$J$5:$J$22),HSTACK(IF('8月30日（日）'!$M$5:$M$22&lt;&gt;"","8/30",""),'8月30日（日）'!$M$5:$M$22,'8月30日（日）'!$L$5:$L$22,'8月30日（日）'!$O$5:$O$22),HSTACK(IF('8月30日（日）'!$R$5:$R$22&lt;&gt;"","8/30",""),'8月30日（日）'!$R$5:$R$22,'8月30日（日）'!$Q$5:$Q$22,'8月30日（日）'!$T$5:$T$22)),FILTER(data,INDEX(data,,2)&lt;&gt;"")),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00808080"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2978,32 +3043,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>担当者リスト</t>
         </is>
       </c>
-      <c r="C1" s="22" t="inlineStr">
+      <c r="C1" s="23" t="inlineStr">
         <is>
           <t>集客経路リスト</t>
         </is>
       </c>
-      <c r="D1" s="22" t="inlineStr">
+      <c r="D1" s="23" t="inlineStr">
         <is>
           <t>集計</t>
         </is>
       </c>
-      <c r="E1" s="23" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>8/28</t>
         </is>
       </c>
-      <c r="F1" s="23" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>8/29</t>
         </is>
       </c>
-      <c r="G1" s="23" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>8/30</t>
         </is>
@@ -3016,15 +3081,15 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="E2" s="24">
+      <c r="E2" s="25">
         <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C2)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C2)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C2)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C2)</f>
         <v/>
       </c>
-      <c r="F2" s="24">
+      <c r="F2" s="25">
         <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C2)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C2)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C2)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C2)</f>
         <v/>
       </c>
-      <c r="G2" s="24">
+      <c r="G2" s="25">
         <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C2)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C2)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C2)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C2)</f>
         <v/>
       </c>
@@ -3040,15 +3105,15 @@
           <t>Googleマップ</t>
         </is>
       </c>
-      <c r="E3" s="24">
+      <c r="E3" s="25">
         <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C3)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C3)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C3)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C3)</f>
         <v/>
       </c>
-      <c r="F3" s="24">
+      <c r="F3" s="25">
         <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C3)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C3)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C3)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C3)</f>
         <v/>
       </c>
-      <c r="G3" s="24">
+      <c r="G3" s="25">
         <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C3)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C3)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C3)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C3)</f>
         <v/>
       </c>
@@ -3064,15 +3129,15 @@
           <t>チラシ</t>
         </is>
       </c>
-      <c r="E4" s="24">
+      <c r="E4" s="25">
         <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C4)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C4)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C4)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C4)</f>
         <v/>
       </c>
-      <c r="F4" s="24">
+      <c r="F4" s="25">
         <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C4)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C4)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C4)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C4)</f>
         <v/>
       </c>
-      <c r="G4" s="24">
+      <c r="G4" s="25">
         <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C4)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C4)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C4)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C4)</f>
         <v/>
       </c>
@@ -3088,15 +3153,15 @@
           <t>紹介</t>
         </is>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="25">
         <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C5)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C5)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C5)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C5)</f>
         <v/>
       </c>
-      <c r="F5" s="24">
+      <c r="F5" s="25">
         <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C5)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C5)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C5)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C5)</f>
         <v/>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="25">
         <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C5)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C5)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C5)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C5)</f>
         <v/>
       </c>
@@ -3112,15 +3177,15 @@
           <t>HP</t>
         </is>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="25">
         <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C6)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C6)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C6)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C6)</f>
         <v/>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="25">
         <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C6)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C6)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C6)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C6)</f>
         <v/>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="25">
         <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C6)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C6)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C6)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C6)</f>
         <v/>
       </c>
@@ -3136,15 +3201,15 @@
           <t>既存会員</t>
         </is>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="25">
         <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C7)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C7)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C7)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C7)</f>
         <v/>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="25">
         <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C7)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C7)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C7)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C7)</f>
         <v/>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="25">
         <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C7)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C7)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C7)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C7)</f>
         <v/>
       </c>
@@ -3155,34 +3220,34 @@
           <t>その他</t>
         </is>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="25">
         <f>COUNTIF('8月28日（金）'!$E$5:$E$22,$C8)+COUNTIF('8月28日（金）'!$J$5:$J$22,$C8)+COUNTIF('8月28日（金）'!$O$5:$O$22,$C8)+COUNTIF('8月28日（金）'!$T$5:$T$22,$C8)</f>
         <v/>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="25">
         <f>COUNTIF('8月29日（土）'!$E$5:$E$22,$C8)+COUNTIF('8月29日（土）'!$J$5:$J$22,$C8)+COUNTIF('8月29日（土）'!$O$5:$O$22,$C8)+COUNTIF('8月29日（土）'!$T$5:$T$22,$C8)</f>
         <v/>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="25">
         <f>COUNTIF('8月30日（日）'!$E$5:$E$22,$C8)+COUNTIF('8月30日（日）'!$J$5:$J$22,$C8)+COUNTIF('8月30日（日）'!$O$5:$O$22,$C8)+COUNTIF('8月30日（日）'!$T$5:$T$22,$C8)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="C9" s="22" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="26">
         <f>SUM(E2:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="25">
+      <c r="F9" s="26">
         <f>SUM(F2:F8)</f>
         <v/>
       </c>
-      <c r="G9" s="25">
+      <c r="G9" s="26">
         <f>SUM(G2:G8)</f>
         <v/>
       </c>

</xml_diff>